<commit_message>
fixes the date matching
</commit_message>
<xml_diff>
--- a/tests/data/regression/carrot_dates.xlsx
+++ b/tests/data/regression/carrot_dates.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Documents/nuh-helper/tests/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Documents/nuh-helper/tests/data/regression/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DEE9836-DF41-EE45-8349-14FDBA4577CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99281EF4-766F-044B-A4A7-784A84B9F8B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19200" yWindow="620" windowWidth="19220" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="observation" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="39">
   <si>
     <t>observation_id</t>
   </si>
@@ -46,9 +46,6 @@
     <t>1</t>
   </si>
   <si>
-    <t>35827394</t>
-  </si>
-  <si>
     <t>1951-12-25</t>
   </si>
   <si>
@@ -61,9 +58,6 @@
     <t>2</t>
   </si>
   <si>
-    <t>35825567</t>
-  </si>
-  <si>
     <t>1981-11-19</t>
   </si>
   <si>
@@ -73,9 +67,6 @@
     <t>3</t>
   </si>
   <si>
-    <t>35826241</t>
-  </si>
-  <si>
     <t>1997-05-11</t>
   </si>
   <si>
@@ -85,9 +76,6 @@
     <t>4</t>
   </si>
   <si>
-    <t>35825531</t>
-  </si>
-  <si>
     <t>1975-06-07</t>
   </si>
   <si>
@@ -115,9 +103,6 @@
     <t>7</t>
   </si>
   <si>
-    <t>35825508</t>
-  </si>
-  <si>
     <t>1956-11-12</t>
   </si>
   <si>
@@ -125,9 +110,6 @@
   </si>
   <si>
     <t>8</t>
-  </si>
-  <si>
-    <t>35827395</t>
   </si>
   <si>
     <t>1985-03-01</t>
@@ -530,237 +512,237 @@
       <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2">
+        <v>27394</v>
+      </c>
+      <c r="D2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
       <c r="F2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3">
+        <v>25567</v>
+      </c>
+      <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>15</v>
-      </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4">
+        <v>26241</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" t="s">
         <v>16</v>
       </c>
-      <c r="B4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" t="s">
-        <v>19</v>
-      </c>
       <c r="F4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
+        <v>17</v>
+      </c>
+      <c r="C5">
+        <v>25531</v>
       </c>
       <c r="D5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E5" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" t="s">
-        <v>8</v>
+        <v>20</v>
+      </c>
+      <c r="C6">
+        <v>27394</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" t="s">
-        <v>13</v>
+        <v>23</v>
+      </c>
+      <c r="C7">
+        <v>25567</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" t="s">
-        <v>31</v>
+        <v>26</v>
+      </c>
+      <c r="C8">
+        <v>25508</v>
       </c>
       <c r="D8" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E8" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="F8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" t="s">
-        <v>35</v>
+        <v>29</v>
+      </c>
+      <c r="C9">
+        <v>27395</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="E9" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="F9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" t="s">
-        <v>8</v>
+        <v>33</v>
+      </c>
+      <c r="C10">
+        <v>27394</v>
       </c>
       <c r="D10" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="E10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" t="s">
-        <v>8</v>
+        <v>36</v>
+      </c>
+      <c r="C11">
+        <v>27394</v>
       </c>
       <c r="D11" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
-      </c>
-      <c r="C12" t="s">
-        <v>17</v>
+        <v>37</v>
+      </c>
+      <c r="C12">
+        <v>26241</v>
       </c>
       <c r="D12" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E12" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" t="s">
-        <v>21</v>
+        <v>38</v>
+      </c>
+      <c r="C13">
+        <v>25531</v>
       </c>
       <c r="D13" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E13" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>